<commit_message>
Updated Issues Tracker Excel spreadsheet with dated entry logs
</commit_message>
<xml_diff>
--- a/BookShelf-App/Docs/BookShelf_Issues_Tracker.xlsx
+++ b/BookShelf-App/Docs/BookShelf_Issues_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\BookShelf-App\BookShelf-App\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01EF42ED-671F-4BB0-9F95-C88E514F69BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16DEA95B-C357-424A-9EA2-92A2A33A7447}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8148" yWindow="648" windowWidth="14892" windowHeight="11592" xr2:uid="{BC64516A-24E3-4AA7-8FE8-B6B3CAE4265A}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="43">
   <si>
     <t>Issue ID:</t>
   </si>
@@ -60,13 +60,121 @@
   </si>
   <si>
     <t>BookShelf Issues Tracker</t>
+  </si>
+  <si>
+    <t>Date Reported:</t>
+  </si>
+  <si>
+    <t>ISSUE-001</t>
+  </si>
+  <si>
+    <t>ISSUE-002</t>
+  </si>
+  <si>
+    <t>ISSUE-003</t>
+  </si>
+  <si>
+    <t>ISSUE-004</t>
+  </si>
+  <si>
+    <t>ISSUE-005</t>
+  </si>
+  <si>
+    <t>ISSUE-006</t>
+  </si>
+  <si>
+    <t>ISSUE-007</t>
+  </si>
+  <si>
+    <t>ISSUE-008</t>
+  </si>
+  <si>
+    <t>ISSUE-009</t>
+  </si>
+  <si>
+    <t>ISSUE-010</t>
+  </si>
+  <si>
+    <t>ISSUE-011</t>
+  </si>
+  <si>
+    <t>ISSUE-012</t>
+  </si>
+  <si>
+    <t>ISSUE-013</t>
+  </si>
+  <si>
+    <t>Solution Structure</t>
+  </si>
+  <si>
+    <t>XAML / Models</t>
+  </si>
+  <si>
+    <t>SQLite DB</t>
+  </si>
+  <si>
+    <t>.NET 9 MAUI</t>
+  </si>
+  <si>
+    <t>Platform / WinUI</t>
+  </si>
+  <si>
+    <t>Version Control</t>
+  </si>
+  <si>
+    <t>Mismatch between physical project folder name (BookShelf-App) and root namespace (BookShelf).</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>RESOLVED</t>
+  </si>
+  <si>
+    <t>Configured &lt;RootNamespace&gt;BookShelf&lt;/RootNamespace&gt; in .csproj to ensure clean namespace declarations without force-renaming local directories.</t>
+  </si>
+  <si>
+    <t>Added helper property CoverUrl with standard fallback placeholder URL in BookSearchItem.cs.</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>Missing cover images (cover_i null) from Open Library API response caused UI rendering errors.</t>
+  </si>
+  <si>
+    <t>App crashed during CreateTableAsync with error: All columns in an index must have the same value for their Unique property.</t>
+  </si>
+  <si>
+    <t>Duplicate window initialization warning in App.xaml.cs when setting MainPage alongside CreateWindow.</t>
+  </si>
+  <si>
+    <t>Platforms/Windows/App.xaml.cs threw CS0103: The name 'MauiProgram' does not exist in current context.</t>
+  </si>
+  <si>
+    <t>Visual Studio background cache files in .vs locked Git from running git add . command.</t>
+  </si>
+  <si>
+    <t>Generated .gitignore file using dotnet new gitignore to exclude .vs, bin, and obj directories prior to initial push.</t>
+  </si>
+  <si>
+    <t>Added using BookShelf; namespace directive to top of Platforms/Windows/App.xaml.cs.</t>
+  </si>
+  <si>
+    <t>Removed legacy MainPage = new AppShell() line from App() constructor to follow .NET 9 lifecycle standards.</t>
+  </si>
+  <si>
+    <t>Removed conflicting [Indexed] attribute from SavedBook.cs (leaving [Unique]) and updated local DB filename to bookshelf_v2.db3 to rebuild clean schema.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -77,6 +185,12 @@
     <font>
       <sz val="16"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -96,7 +210,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -109,59 +223,67 @@
         <color theme="3" tint="0.749992370372631"/>
       </left>
       <right/>
-      <top style="thin">
-        <color theme="3" tint="0.749992370372631"/>
-      </top>
-      <bottom style="thin">
-        <color theme="3" tint="0.749992370372631"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="3" tint="0.749992370372631"/>
-      </top>
-      <bottom style="thin">
-        <color theme="3" tint="0.749992370372631"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color theme="3" tint="0.749992370372631"/>
-      </right>
-      <top style="thin">
-        <color theme="3" tint="0.749992370372631"/>
-      </top>
-      <bottom style="thin">
-        <color theme="3" tint="0.749992370372631"/>
-      </bottom>
+      <top/>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="9">
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -175,15 +297,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{51914C63-0C41-4065-82EE-13A72D1607F1}" name="Table1" displayName="Table1" ref="B6:G38" totalsRowShown="0">
-  <autoFilter ref="B6:G38" xr:uid="{51914C63-0C41-4065-82EE-13A72D1607F1}"/>
-  <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{CD283CCF-C7A0-4753-86D1-DA6AEE50145C}" name="Issue ID:"/>
-    <tableColumn id="2" xr3:uid="{091F31E0-5637-47DF-A494-4F36A6B696C9}" name="Component:"/>
-    <tableColumn id="3" xr3:uid="{33B3E06B-8F5D-4909-A91A-6F0887339523}" name="Description:"/>
-    <tableColumn id="4" xr3:uid="{B0CCE9D0-0183-4FDF-9B9E-3F5F31DD8297}" name="Severity:"/>
-    <tableColumn id="5" xr3:uid="{DE842D55-EBE6-4621-9F49-2AE98963D504}" name="Status:"/>
-    <tableColumn id="6" xr3:uid="{0B610FCF-74ED-46DA-A382-1FD294E26944}" name="Resolution:"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{51914C63-0C41-4065-82EE-13A72D1607F1}" name="Table1" displayName="Table1" ref="B6:H38" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
+  <autoFilter ref="B6:H38" xr:uid="{51914C63-0C41-4065-82EE-13A72D1607F1}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{CD283CCF-C7A0-4753-86D1-DA6AEE50145C}" name="Issue ID:" dataDxfId="8"/>
+    <tableColumn id="7" xr3:uid="{37DB08C9-B734-41D2-8A41-6494A3BF4AE9}" name="Date Reported:" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{091F31E0-5637-47DF-A494-4F36A6B696C9}" name="Component:" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{33B3E06B-8F5D-4909-A91A-6F0887339523}" name="Description:" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{B0CCE9D0-0183-4FDF-9B9E-3F5F31DD8297}" name="Severity:" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{DE842D55-EBE6-4621-9F49-2AE98963D504}" name="Status:" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{0B610FCF-74ED-46DA-A382-1FD294E26944}" name="Resolution:" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -506,16 +629,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9616B9B9-A3D6-4BBA-871C-D6E138B3D2A0}">
-  <dimension ref="B3:G6"/>
+  <dimension ref="B3:H19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="9.88671875" customWidth="1"/>
-    <col min="3" max="4" width="13.109375" customWidth="1"/>
-    <col min="5" max="5" width="10.21875" customWidth="1"/>
-    <col min="7" max="7" width="12.21875" customWidth="1"/>
+    <col min="1" max="1" width="8.88671875" style="1"/>
+    <col min="2" max="2" width="12.5546875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="17.109375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="20.5546875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="36.5546875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="13.109375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="12.21875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="43.88671875" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:7" ht="21" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:8" ht="21" x14ac:dyDescent="0.3">
       <c r="B3" s="2" t="s">
         <v>6</v>
       </c>
@@ -523,35 +651,213 @@
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
-      <c r="G3" s="4"/>
-    </row>
-    <row r="4" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B4" s="1"/>
-    </row>
-    <row r="6" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B6" t="s">
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+    </row>
+    <row r="4" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B4" s="4"/>
+    </row>
+    <row r="6" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B6" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" s="1" t="s">
         <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="2:8" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="B7" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" s="5">
+        <v>46260</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B8" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="6">
+        <v>46260</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9" spans="2:8" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="B9" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" s="6">
+        <v>46260</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="10" spans="2:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B10" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" s="6">
+        <v>46260</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="11" spans="2:8" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="B11" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" s="6">
+        <v>46260</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="12" spans="2:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B12" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C12" s="6">
+        <v>46260</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="13" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B13" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B14" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B15" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="16" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B16" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B17" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="18" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B18" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="19" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B19" s="1" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B3:G3"/>
+    <mergeCell ref="B3:H3"/>
   </mergeCells>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>

<commit_message>
Updated TC-03 severity rating to High and logged retest details
</commit_message>
<xml_diff>
--- a/BookShelf-App/Docs/BookShelf_Issues_Tracker.xlsx
+++ b/BookShelf-App/Docs/BookShelf_Issues_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\BookShelf-App\BookShelf-App\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16DEA95B-C357-424A-9EA2-92A2A33A7447}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D258B0DF-FF26-4DE7-91EE-9A52D22F1550}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8148" yWindow="648" windowWidth="14892" windowHeight="11592" xr2:uid="{BC64516A-24E3-4AA7-8FE8-B6B3CAE4265A}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="47">
   <si>
     <t>Issue ID:</t>
   </si>
@@ -168,13 +168,88 @@
   </si>
   <si>
     <t>Removed conflicting [Indexed] attribute from SavedBook.cs (leaving [Unique]) and updated local DB filename to bookshelf_v2.db3 to rebuild clean schema.</t>
+  </si>
+  <si>
+    <t>SQLite Database</t>
+  </si>
+  <si>
+    <t>Save book from Search view to local collection and verify table creation.</t>
+  </si>
+  <si>
+    <t>PASS (Retested)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Initial Run FAILED</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: CreateTableAsync threw System.Exception due to duplicate [Unique] &amp; [Indexed] attributes on OpenLibraryKey.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>FIX</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: Removed [Indexed] attribute &amp; reset database schema. Retest </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PASSED</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -183,7 +258,22 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="16"/>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -191,6 +281,30 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -231,25 +345,43 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -257,30 +389,140 @@
   </cellStyles>
   <dxfs count="9">
     <dxf>
+      <font>
+        <b/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <font>
+        <b/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
@@ -297,16 +539,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{51914C63-0C41-4065-82EE-13A72D1607F1}" name="Table1" displayName="Table1" ref="B6:H38" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{51914C63-0C41-4065-82EE-13A72D1607F1}" name="Table1" displayName="Table1" ref="B6:H38" totalsRowShown="0" headerRowDxfId="8" dataDxfId="2">
   <autoFilter ref="B6:H38" xr:uid="{51914C63-0C41-4065-82EE-13A72D1607F1}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{CD283CCF-C7A0-4753-86D1-DA6AEE50145C}" name="Issue ID:" dataDxfId="8"/>
-    <tableColumn id="7" xr3:uid="{37DB08C9-B734-41D2-8A41-6494A3BF4AE9}" name="Date Reported:" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{091F31E0-5637-47DF-A494-4F36A6B696C9}" name="Component:" dataDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{33B3E06B-8F5D-4909-A91A-6F0887339523}" name="Description:" dataDxfId="5"/>
-    <tableColumn id="4" xr3:uid="{B0CCE9D0-0183-4FDF-9B9E-3F5F31DD8297}" name="Severity:" dataDxfId="4"/>
-    <tableColumn id="5" xr3:uid="{DE842D55-EBE6-4621-9F49-2AE98963D504}" name="Status:" dataDxfId="3"/>
-    <tableColumn id="6" xr3:uid="{0B610FCF-74ED-46DA-A382-1FD294E26944}" name="Resolution:" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{CD283CCF-C7A0-4753-86D1-DA6AEE50145C}" name="Issue ID:" dataDxfId="0"/>
+    <tableColumn id="7" xr3:uid="{37DB08C9-B734-41D2-8A41-6494A3BF4AE9}" name="Date Reported:" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{091F31E0-5637-47DF-A494-4F36A6B696C9}" name="Component:" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{33B3E06B-8F5D-4909-A91A-6F0887339523}" name="Description:" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{B0CCE9D0-0183-4FDF-9B9E-3F5F31DD8297}" name="Severity:" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{DE842D55-EBE6-4621-9F49-2AE98963D504}" name="Status:" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{0B610FCF-74ED-46DA-A382-1FD294E26944}" name="Resolution:" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -629,7 +871,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9616B9B9-A3D6-4BBA-871C-D6E138B3D2A0}">
-  <dimension ref="B3:H19"/>
+  <dimension ref="B3:H38"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="1"/>
@@ -638,226 +880,451 @@
     <col min="4" max="4" width="20.5546875" style="1" customWidth="1"/>
     <col min="5" max="5" width="36.5546875" style="1" customWidth="1"/>
     <col min="6" max="6" width="13.109375" style="1" customWidth="1"/>
-    <col min="7" max="7" width="12.21875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="12.21875" style="3" customWidth="1"/>
     <col min="8" max="8" width="43.88671875" style="1" customWidth="1"/>
     <col min="9" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:8" ht="21" x14ac:dyDescent="0.3">
-      <c r="B3" s="2" t="s">
+    <row r="3" spans="2:8" s="12" customFormat="1" ht="23.4" x14ac:dyDescent="0.3">
+      <c r="B3" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
+      <c r="C3" s="11"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="11"/>
+      <c r="F3" s="11"/>
+      <c r="G3" s="11"/>
+      <c r="H3" s="11"/>
     </row>
     <row r="4" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B4" s="4"/>
-    </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B6" s="1" t="s">
+      <c r="B4" s="2"/>
+    </row>
+    <row r="6" spans="2:8" s="6" customFormat="1" ht="18" x14ac:dyDescent="0.3">
+      <c r="B6" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="G6" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="H6" s="6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="2:8" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B7" s="1" t="s">
+    <row r="7" spans="2:8" ht="78" x14ac:dyDescent="0.3">
+      <c r="B7" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C7" s="8">
         <v>46260</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="D7" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="E7" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="F7" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="G7" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="H7" s="1" t="s">
+      <c r="H7" s="4" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="2:8" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B8" s="1" t="s">
+    <row r="8" spans="2:8" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="B8" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="6">
+      <c r="C8" s="9">
         <v>46260</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="D8" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="E8" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="F8" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c r="G8" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="H8" s="1" t="s">
+      <c r="H8" s="4" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="2:8" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B9" s="1" t="s">
+    <row r="9" spans="2:8" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="B9" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="6">
+      <c r="C9" s="9">
         <v>46260</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="D9" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="E9" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="F9" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="G9" s="1" t="s">
+      <c r="G9" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="H9" s="1" t="s">
+      <c r="H9" s="4" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="2:8" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B10" s="1" t="s">
+    <row r="10" spans="2:8" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="B10" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C10" s="6">
+      <c r="C10" s="9">
         <v>46260</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="D10" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="E10" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="F10" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="G10" s="1" t="s">
+      <c r="G10" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="H10" s="1" t="s">
+      <c r="H10" s="4" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="11" spans="2:8" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B11" s="1" t="s">
+    <row r="11" spans="2:8" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="B11" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C11" s="6">
+      <c r="C11" s="9">
         <v>46260</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="D11" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="E11" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="F11" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="G11" s="1" t="s">
+      <c r="G11" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="H11" s="1" t="s">
+      <c r="H11" s="4" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="12" spans="2:8" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B12" s="1" t="s">
+    <row r="12" spans="2:8" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="B12" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C12" s="6">
+      <c r="C12" s="9">
         <v>46260</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="D12" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="E12" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="F12" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="G12" s="1" t="s">
+      <c r="G12" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="H12" s="1" t="s">
+      <c r="H12" s="4" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B13" s="1" t="s">
+    <row r="13" spans="2:8" ht="93.6" x14ac:dyDescent="0.3">
+      <c r="B13" s="5" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B14" s="1" t="s">
+      <c r="C13" s="9">
+        <v>46260</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="14" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B14" s="5" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B15" s="1" t="s">
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
+      <c r="F14" s="4"/>
+      <c r="G14" s="5"/>
+      <c r="H14" s="4"/>
+    </row>
+    <row r="15" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B15" s="5" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="16" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B16" s="1" t="s">
+      <c r="C15" s="4"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+      <c r="F15" s="4"/>
+      <c r="G15" s="5"/>
+      <c r="H15" s="4"/>
+    </row>
+    <row r="16" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B16" s="5" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B17" s="1" t="s">
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
+      <c r="F16" s="4"/>
+      <c r="G16" s="5"/>
+      <c r="H16" s="4"/>
+    </row>
+    <row r="17" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B17" s="5" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B18" s="1" t="s">
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+      <c r="F17" s="4"/>
+      <c r="G17" s="5"/>
+      <c r="H17" s="4"/>
+    </row>
+    <row r="18" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B18" s="5" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B19" s="1" t="s">
+      <c r="C18" s="4"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
+      <c r="F18" s="4"/>
+      <c r="G18" s="5"/>
+      <c r="H18" s="4"/>
+    </row>
+    <row r="19" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B19" s="5" t="s">
         <v>20</v>
       </c>
+      <c r="C19" s="4"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
+      <c r="F19" s="4"/>
+      <c r="G19" s="5"/>
+      <c r="H19" s="4"/>
+    </row>
+    <row r="20" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B20" s="5"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+      <c r="F20" s="4"/>
+      <c r="G20" s="5"/>
+      <c r="H20" s="4"/>
+    </row>
+    <row r="21" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B21" s="5"/>
+      <c r="C21" s="4"/>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4"/>
+      <c r="F21" s="4"/>
+      <c r="G21" s="5"/>
+      <c r="H21" s="4"/>
+    </row>
+    <row r="22" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B22" s="5"/>
+      <c r="C22" s="4"/>
+      <c r="D22" s="4"/>
+      <c r="E22" s="4"/>
+      <c r="F22" s="4"/>
+      <c r="G22" s="5"/>
+      <c r="H22" s="4"/>
+    </row>
+    <row r="23" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B23" s="5"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="4"/>
+      <c r="F23" s="4"/>
+      <c r="G23" s="5"/>
+      <c r="H23" s="4"/>
+    </row>
+    <row r="24" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B24" s="5"/>
+      <c r="C24" s="4"/>
+      <c r="D24" s="4"/>
+      <c r="E24" s="4"/>
+      <c r="F24" s="4"/>
+      <c r="G24" s="5"/>
+      <c r="H24" s="4"/>
+    </row>
+    <row r="25" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B25" s="5"/>
+      <c r="C25" s="4"/>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4"/>
+      <c r="F25" s="4"/>
+      <c r="G25" s="5"/>
+      <c r="H25" s="4"/>
+    </row>
+    <row r="26" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B26" s="5"/>
+      <c r="C26" s="4"/>
+      <c r="D26" s="4"/>
+      <c r="E26" s="4"/>
+      <c r="F26" s="4"/>
+      <c r="G26" s="5"/>
+      <c r="H26" s="4"/>
+    </row>
+    <row r="27" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B27" s="5"/>
+      <c r="C27" s="4"/>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4"/>
+      <c r="F27" s="4"/>
+      <c r="G27" s="5"/>
+      <c r="H27" s="4"/>
+    </row>
+    <row r="28" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B28" s="5"/>
+      <c r="C28" s="4"/>
+      <c r="D28" s="4"/>
+      <c r="E28" s="4"/>
+      <c r="F28" s="4"/>
+      <c r="G28" s="5"/>
+      <c r="H28" s="4"/>
+    </row>
+    <row r="29" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B29" s="5"/>
+      <c r="C29" s="4"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4"/>
+      <c r="F29" s="4"/>
+      <c r="G29" s="5"/>
+      <c r="H29" s="4"/>
+    </row>
+    <row r="30" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B30" s="5"/>
+      <c r="C30" s="4"/>
+      <c r="D30" s="4"/>
+      <c r="E30" s="4"/>
+      <c r="F30" s="4"/>
+      <c r="G30" s="5"/>
+      <c r="H30" s="4"/>
+    </row>
+    <row r="31" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B31" s="5"/>
+      <c r="C31" s="4"/>
+      <c r="D31" s="4"/>
+      <c r="E31" s="4"/>
+      <c r="F31" s="4"/>
+      <c r="G31" s="5"/>
+      <c r="H31" s="4"/>
+    </row>
+    <row r="32" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B32" s="5"/>
+      <c r="C32" s="4"/>
+      <c r="D32" s="4"/>
+      <c r="E32" s="4"/>
+      <c r="F32" s="4"/>
+      <c r="G32" s="5"/>
+      <c r="H32" s="4"/>
+    </row>
+    <row r="33" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B33" s="5"/>
+      <c r="C33" s="4"/>
+      <c r="D33" s="4"/>
+      <c r="E33" s="4"/>
+      <c r="F33" s="4"/>
+      <c r="G33" s="5"/>
+      <c r="H33" s="4"/>
+    </row>
+    <row r="34" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B34" s="5"/>
+      <c r="C34" s="4"/>
+      <c r="D34" s="4"/>
+      <c r="E34" s="4"/>
+      <c r="F34" s="4"/>
+      <c r="G34" s="5"/>
+      <c r="H34" s="4"/>
+    </row>
+    <row r="35" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B35" s="5"/>
+      <c r="C35" s="4"/>
+      <c r="D35" s="4"/>
+      <c r="E35" s="4"/>
+      <c r="F35" s="4"/>
+      <c r="G35" s="5"/>
+      <c r="H35" s="4"/>
+    </row>
+    <row r="36" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B36" s="5"/>
+      <c r="C36" s="4"/>
+      <c r="D36" s="4"/>
+      <c r="E36" s="4"/>
+      <c r="F36" s="4"/>
+      <c r="G36" s="5"/>
+      <c r="H36" s="4"/>
+    </row>
+    <row r="37" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B37" s="5"/>
+      <c r="C37" s="4"/>
+      <c r="D37" s="4"/>
+      <c r="E37" s="4"/>
+      <c r="F37" s="4"/>
+      <c r="G37" s="5"/>
+      <c r="H37" s="4"/>
+    </row>
+    <row r="38" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B38" s="5"/>
+      <c r="C38" s="4"/>
+      <c r="D38" s="4"/>
+      <c r="E38" s="4"/>
+      <c r="F38" s="4"/>
+      <c r="G38" s="5"/>
+      <c r="H38" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="B3:H3"/>
   </mergeCells>
-  <phoneticPr fontId="2" type="noConversion"/>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>

<commit_message>
Updated Issues Tracker (ISSUE-008 to ISSUE-011) and Test Plan (TC-05 to TC-10) with extension resolutions
</commit_message>
<xml_diff>
--- a/BookShelf-App/Docs/BookShelf_Issues_Tracker.xlsx
+++ b/BookShelf-App/Docs/BookShelf_Issues_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\BookShelf-App\BookShelf-App\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D258B0DF-FF26-4DE7-91EE-9A52D22F1550}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFE6BA70-F9A6-4A86-A752-4A5B39062D8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8148" yWindow="648" windowWidth="14892" windowHeight="11592" xr2:uid="{BC64516A-24E3-4AA7-8FE8-B6B3CAE4265A}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="59">
   <si>
     <t>Issue ID:</t>
   </si>
@@ -243,6 +243,42 @@
       </rPr>
       <t>.</t>
     </r>
+  </si>
+  <si>
+    <t>XAML / Border Control</t>
+  </si>
+  <si>
+    <t>XAML / Image Aspect</t>
+  </si>
+  <si>
+    <t>UI / Event Handling</t>
+  </si>
+  <si>
+    <t>SQLite / Persistence</t>
+  </si>
+  <si>
+    <t>CornerRadius property not found on &lt;Border&gt; (XLS0413 / XC0009).</t>
+  </si>
+  <si>
+    <t>Invalid enum value AspectScaleToFit on &lt;Image&gt; (XLS0413 / XC0007).</t>
+  </si>
+  <si>
+    <t>MyBooksPage froze on Windows due to an infinite re-entrancy loop during picker/filter updates.</t>
+  </si>
+  <si>
+    <t>Reading status, star ratings, and personal notes reset when toggling between tab pages.</t>
+  </si>
+  <si>
+    <t>Replaced direct CornerRadius attribute with nested &lt;Border.StrokeShape&gt;&lt;RoundRectangle CornerRadius="8"/&gt;&lt;/Border.StrokeShape&gt;.</t>
+  </si>
+  <si>
+    <t>Updated attribute value to valid MAUI enum Aspect="AspectFit".</t>
+  </si>
+  <si>
+    <t>Added boolean _isUpdating guard flag in MyBooksPage.xaml.cs to prevent recursive event firing during data binding.</t>
+  </si>
+  <si>
+    <t>Refactored SaveBookAsync to check book.Id != 0, called UpdateBookAsync explicitly on UI changes, and added Mode=TwoWay to XAML picker bindings.</t>
   </si>
 </sst>
 </file>
@@ -927,7 +963,7 @@
         <v>8</v>
       </c>
       <c r="C7" s="8">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>21</v>
@@ -950,7 +986,7 @@
         <v>9</v>
       </c>
       <c r="C8" s="9">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="D8" s="4" t="s">
         <v>22</v>
@@ -972,8 +1008,8 @@
       <c r="B9" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="9">
-        <v>46260</v>
+      <c r="C9" s="8">
+        <v>46261</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>23</v>
@@ -996,7 +1032,7 @@
         <v>11</v>
       </c>
       <c r="C10" s="9">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="D10" s="4" t="s">
         <v>24</v>
@@ -1018,8 +1054,8 @@
       <c r="B11" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C11" s="9">
-        <v>46260</v>
+      <c r="C11" s="8">
+        <v>46261</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>25</v>
@@ -1042,7 +1078,7 @@
         <v>13</v>
       </c>
       <c r="C12" s="9">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="D12" s="4" t="s">
         <v>26</v>
@@ -1064,8 +1100,8 @@
       <c r="B13" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C13" s="9">
-        <v>46260</v>
+      <c r="C13" s="8">
+        <v>46261</v>
       </c>
       <c r="D13" s="4" t="s">
         <v>43</v>
@@ -1083,49 +1119,97 @@
         <v>46</v>
       </c>
     </row>
-    <row r="14" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:8" ht="62.4" x14ac:dyDescent="0.3">
       <c r="B14" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="5"/>
-      <c r="H14" s="4"/>
-    </row>
-    <row r="15" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="C14" s="8">
+        <v>46262</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G14" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="15" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B15" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C15" s="4"/>
-      <c r="D15" s="4"/>
-      <c r="E15" s="4"/>
-      <c r="F15" s="4"/>
-      <c r="G15" s="5"/>
-      <c r="H15" s="4"/>
-    </row>
-    <row r="16" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="C15" s="8">
+        <v>46262</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G15" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="16" spans="2:8" ht="46.8" x14ac:dyDescent="0.3">
       <c r="B16" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
-      <c r="E16" s="4"/>
-      <c r="F16" s="4"/>
-      <c r="G16" s="5"/>
-      <c r="H16" s="4"/>
-    </row>
-    <row r="17" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="C16" s="8">
+        <v>46262</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="G16" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="17" spans="2:8" ht="62.4" x14ac:dyDescent="0.3">
       <c r="B17" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C17" s="4"/>
-      <c r="D17" s="4"/>
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
-      <c r="G17" s="5"/>
-      <c r="H17" s="4"/>
+      <c r="C17" s="8">
+        <v>46262</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="G17" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H17" s="4" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="18" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B18" s="5" t="s">

</xml_diff>